<commit_message>
docs(tools-sync): Watchlist_Ersatzbank_Monitor SSoT-Sync — SNPS/SPGI/FICO Scores + Header
Letzte unsynchronisierte SSoT-Drift-Quelle nach KONTEXT/Faktortabelle-Reconcile
heute (`db66d99`). Stand der XLSX war 15.04.2026 — 12 Tage stale.

8 Cells geändert:
- Header + QuickScreen-Header: Stand 15.04. → 27.04.
- SNPS Score 79→76 (DEFCON v3.5 Audit 16.04., Goodwill-Malus Ansys)
- SPGI Score 79→74 (M&A-Goodwill IHS Markit, Non-GAAP ROIC ~82)
- FICO Score 70→67 (TTM-Kurscrash-Verzerrung)
- QuickScreen-Nächster-Schritt-Spalten für die 3 Tickers angepasst

Markt-Drift in Tabellen-P/FCF/ROIC-Werten ([KB]-Snapshots) bewusst NICHT
angepasst — XLSX ist Snapshot-Format, kein Live-Feed. Quick-Screener-Sweep
27.04. zeigte Multiple-Drift bei AVGO/NVDA/VEEV/FICO, aber Score-Logik intakt.

Satelliten_Monitor v2.0 (Stand 23.04.) ist bereits konsistent — alle 11
Live-Scores match PORTFOLIO.md, Sparraten-Summe 285€ ✓. Kein Edit nötig.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03_Tools/Watchlist_Ersatzbank_Monitor_v1.1.xlsx
+++ b/03_Tools/Watchlist_Ersatzbank_Monitor_v1.1.xlsx
@@ -928,7 +928,7 @@
     <row r="1" ht="21.95" customHeight="1" s="67">
       <c r="A1" s="80" t="inlineStr">
         <is>
-          <t>🦅  DYNASTIEDEPOT – WATCHLIST / ERSATZBANK MONITOR v1.1  |  Stand: 15.04.2026</t>
+          <t>🦅  DYNASTIEDEPOT – WATCHLIST / ERSATZBANK MONITOR v1.1  |  Stand: 27.04.2026</t>
         </is>
       </c>
     </row>
@@ -1697,7 +1697,7 @@
       </c>
       <c r="L13" s="39" t="inlineStr">
         <is>
-          <t>79 / DEFCON 3</t>
+          <t>76 / DEFCON 3</t>
         </is>
       </c>
       <c r="M13" s="40" t="inlineStr">
@@ -1707,7 +1707,7 @@
       </c>
       <c r="N13" s="41" t="inlineStr">
         <is>
-          <t>P/FCF ~32x 🟢. Wide Moat [KB] 18/20. Score 79 — 1 Pkt unter 80-Schwelle. Re-Analyse Q1 Earnings 28.04.2026.</t>
+          <t>P/FCF ~32x 🟢. Wide Moat [KB] 18/20. Score 76 (post-DEFCON v3.5 Audit 16.04.2026: 79→76, Goodwill-Malus Ansys-Akquisition -3 Pkt). Re-Analyse Q1 Earnings 28.04.2026.</t>
         </is>
       </c>
       <c r="O13" s="42" t="inlineStr">
@@ -1851,7 +1851,7 @@
       </c>
       <c r="L15" s="39" t="inlineStr">
         <is>
-          <t>79 / DEFCON 3</t>
+          <t>74 / DEFCON 3</t>
         </is>
       </c>
       <c r="M15" s="40" t="inlineStr">
@@ -1861,7 +1861,7 @@
       </c>
       <c r="N15" s="41" t="inlineStr">
         <is>
-          <t>P/FCF ~22x 🟢. Wide Moat 19/20. Ratings-Duopol. Earnings 28.04.2026 → Katalysator. Re-Analyse bei Score ≥80.</t>
+          <t>P/FCF ~22x 🟢. Wide Moat 19/20. Ratings-Duopol. Score 74 (post-DEFCON v3.5 Audit 16.04.2026: 77→74, ROIC-Verzerrung durch IHS Markit M&amp;A-Goodwill, Non-GAAP ~82). Earnings 28.04.2026 → Katalysator. Re-Analyse bei Score ≥80.</t>
         </is>
       </c>
       <c r="O15" s="42" t="inlineStr">
@@ -2236,7 +2236,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>70 / DEFCON 3</t>
+          <t>67 / DEFCON 3</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -2246,7 +2246,7 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Vollanalyse 03.04.2026. Score 70 / DEFCON 3. Fwd P/FCF ~19x 🟢 (nach -52% Crash). ROIC 75% exzellent. 10b5-1 Cashless-Exercise erkannt. Re-Analyse bei VEEV-Schwäche.</t>
+          <t>Vollanalyse 03.04.2026. Score 67 (post-DEFCON v3.5 Audit 16.04.2026: 70→67, TTM-Verzerrung Kurscrash -52%). Fwd P/FCF ~19x 🟢. ROIC 75% exzellent. Quick-Screener-Sweep 27.04.2026: ROIC 42-45% TTM bestätigt, weiterer Kursfall -48% YTD trotz +40% EPS-Growth = Multiple-Compression.</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
@@ -2262,7 +2262,7 @@
     <row r="23" ht="15.95" customHeight="1" s="67">
       <c r="A23" s="62" t="inlineStr">
         <is>
-          <t>⚡  QuickScreen Ergebnis – 15.04.2026  |  Filter: P/FCF ≤35🟢/≤45🟡/&gt;45🔴  |  ROIC ≥15%🟢/≥12%🟡/&lt;12%🔴  |  Moat Wide🟢/Narrow🟡/None🔴</t>
+          <t>⚡  QuickScreen Ergebnis – 27.04.2026  |  Filter: P/FCF ≤35🟢/≤45🟡/&gt;45🔴  |  ROIC ≥15%🟢/≥12%🟡/&lt;12%🔴  |  Moat Wide🟢/Narrow🟡/None🔴</t>
         </is>
       </c>
     </row>
@@ -2472,7 +2472,7 @@
       </c>
       <c r="H28" s="51" t="inlineStr">
         <is>
-          <t>Score 79. 1 Pkt unter 80-Schwelle. Re-Analyse Mai 2026.</t>
+          <t>Score 76 (post-v3.5 Audit). 4 Pkt unter 80-Schwelle. Re-Analyse Q1 Earnings 28.04.2026.</t>
         </is>
       </c>
     </row>
@@ -2514,7 +2514,7 @@
       </c>
       <c r="H29" s="51" t="inlineStr">
         <is>
-          <t>Score 79. Earnings 28.04.2026 → Katalysator-Check.</t>
+          <t>Score 74 (post-v3.5 Audit). Earnings 28.04.2026 → Katalysator-Check.</t>
         </is>
       </c>
     </row>
@@ -2976,7 +2976,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Score 70 / DEFCON 3. Fwd P/FCF ~19x 🟢. ROIC 75% exzellent. Re-Analyse bei VEEV-Schwäche.</t>
+          <t>Score 67 / DEFCON 3 (post-v3.5 Audit). Fwd P/FCF ~19x 🟢. ROIC 75% exzellent. Re-Analyse bei VEEV-Schwäche.</t>
         </is>
       </c>
     </row>

</xml_diff>